<commit_message>
Import template: remove FUOYE from the example notes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013SUeaNcyeUTPoKBLAPaRiT
</commit_message>
<xml_diff>
--- a/public/templates/university-import-template.xlsx
+++ b/public/templates/university-import-template.xlsx
@@ -546,7 +546,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Short code, e.g. UI, UNILAG, FUOYE. A new code creates a new university.</t>
+          <t>Short code, e.g. UI or UNILAG. A new code creates a new university.</t>
         </is>
       </c>
     </row>
@@ -675,7 +675,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Optional: points added for one sitting (FUOYE uses 10).</t>
+          <t>Optional: points added to the aggregate for one O'Level sitting. Blank = none.</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Optional: points added for two sittings (FUOYE uses 6).</t>
+          <t>Optional: points added for two sittings. Fill in both bonus rows, or neither.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Import template: dropdowns and validation
University sheet: dropdowns for code and location state; number checks on
weightings, max scores, Post-UTME minimum, two-sitting deduction, sitting
bonus and quotas. Courses sheet: faculty and minimum-credits dropdowns;
cut-off cells accept 0-100 (JAMB 0-400), 'none' or blank. Lists live on a
hidden third sheet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013SUeaNcyeUTPoKBLAPaRiT
</commit_message>
<xml_diff>
--- a/public/templates/university-import-template.xlsx
+++ b/public/templates/university-import-template.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="University" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Courses" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -775,6 +776,38 @@
       <c r="C19" s="3" t="n"/>
     </row>
   </sheetData>
+  <dataValidations count="8">
+    <dataValidation sqref="B2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="University code" error="Pick an existing code to update it, or type a new code to create a university." promptTitle="University code" prompt="Pick an existing code to update it, or type a new code to create a university." type="list" errorStyle="warning">
+      <formula1>=Lists!$C$2:$C$7</formula1>
+    </dataValidation>
+    <dataValidation sqref="B4" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="State" error="Choose the state the university is in." promptTitle="State" prompt="Choose the state the university is in." type="list" errorStyle="stop">
+      <formula1>=Lists!$A$2:$A$38</formula1>
+    </dataValidation>
+    <dataValidation sqref="B5:B7" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Weighting" error="A percentage from 0 to 100. UTME + Post-UTME + O'Level (+ sitting bonus) must total 100." promptTitle="Weighting" prompt="A percentage from 0 to 100. UTME + Post-UTME + O'Level (+ sitting bonus) must total 100." type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>100</formula2>
+    </dataValidation>
+    <dataValidation sqref="B8:B9" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Maximum score" error="The highest possible score, e.g. 400 for UTME, 100 for Post-UTME." promptTitle="Maximum score" prompt="The highest possible score, e.g. 400 for UTME, 100 for Post-UTME." type="decimal" operator="between">
+      <formula1>1</formula1>
+      <formula2>1000</formula2>
+    </dataValidation>
+    <dataValidation sqref="B10" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Post-UTME minimum" error="Optional percentage. Leave blank if there's no minimum." promptTitle="Post-UTME minimum" prompt="Optional percentage. Leave blank if there's no minimum." type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>100</formula2>
+    </dataValidation>
+    <dataValidation sqref="B11" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Two-sitting deduction" error="Optional O'Level points deducted for two sittings. Leave blank if none." promptTitle="Two-sitting deduction" prompt="Optional O'Level points deducted for two sittings. Leave blank if none." type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>30</formula2>
+    </dataValidation>
+    <dataValidation sqref="B12:B13" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Sitting bonus" error="Optional points. Fill in both bonus rows, or leave both blank." promptTitle="Sitting bonus" prompt="Optional points. Fill in both bonus rows, or leave both blank." type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>100</formula2>
+    </dataValidation>
+    <dataValidation sqref="B17:B19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Quota" error="A percentage. Merit + catchment + ELDS quotas must total 100." promptTitle="Quota" prompt="A percentage. Merit + catchment + ELDS quotas must total 100." type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>100</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2242,7 +2275,422 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="6">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Faculty" error="Choose a faculty. You can type a new one if this university has a faculty not listed." promptTitle="Faculty" prompt="Choose a faculty. You can type a new one if this university has a faculty not listed." type="list" errorStyle="warning">
+      <formula1>=Lists!$B$2:$B$9</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Minimum credits" error="Number of O'Level credits required (usually 5)." promptTitle="Minimum credits" prompt="Number of O'Level credits required (usually 5)." type="list" errorStyle="stop">
+      <formula1>=Lists!$D$2:$D$11</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Merit cut-off" error="Enter a number from 0 to 100, the word none to clear it, or leave blank to keep the current value." promptTitle="Merit cut-off" prompt="0–100. Blank = keep current; none = clear." type="custom">
+      <formula1>=OR(I2="",LOWER(I2)="none",AND(ISNUMBER(I2),I2&gt;=0,I2&lt;=100))</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Catchment cut-off" error="Enter a number from 0 to 100, the word none to clear it, or leave blank to keep the current value." promptTitle="Catchment cut-off" prompt="0–100. Blank = keep current; none = clear." type="custom">
+      <formula1>=OR(J2="",LOWER(J2)="none",AND(ISNUMBER(J2),J2&gt;=0,J2&lt;=100))</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="ELDS cut-off" error="Enter a number from 0 to 100, the word none to clear it, or leave blank to keep the current value." promptTitle="ELDS cut-off" prompt="0–100. Blank = keep current; none = clear." type="custom">
+      <formula1>=OR(K2="",LOWER(K2)="none",AND(ISNUMBER(K2),K2&gt;=0,K2&lt;=100))</formula1>
+    </dataValidation>
+    <dataValidation sqref="L2:L500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="JAMB cut-off" error="Enter a number from 0 to 400, the word none to clear it, or leave blank to keep the current value." promptTitle="JAMB cut-off" prompt="0–400. Blank = keep current; none = clear." type="custom">
+      <formula1>=OR(L2="",LOWER(L2)="none",AND(ISNUMBER(L2),L2&gt;=0,L2&lt;=400))</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>states</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>faculties</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>codes</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>credits</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Abia</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Clinical Sciences</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Adamawa</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Law</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>UNILAG</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Akwa Ibom</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Engineering &amp; Technology</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>OAU</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Anambra</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Arts</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>FUTA</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Bauchi</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Social &amp; Management Sciences</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>FUNAAB</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bayelsa</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Science</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>FUOYE</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Benue</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Borno</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Logistics &amp; Innovation Technology</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Cross River</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Delta</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Ebonyi</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Edo</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Ekiti</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Enugu</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Gombe</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Imo</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Jigawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Kaduna</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Kano</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Katsina</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Kebbi</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Kogi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Kwara</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Lagos</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Nasarawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Niger</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Ogun</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Ondo</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Osun</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Oyo</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Plateau</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Rivers</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Sokoto</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Taraba</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Yobe</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Zamfara</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>FCT (Abuja)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>